<commit_message>
add : change api export, import imployee to map BeStaffDate and BeTviecDate
</commit_message>
<xml_diff>
--- a/aspnet-core/src/HRMv2.Web.Host/wwwroot/template/Create-Employees.xlsx
+++ b/aspnet-core/src/HRMv2.Web.Host/wwwroot/template/Create-Employees.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work2\ncc-erp-hrm-v2\aspnet-core\src\HRMv2.Web.Host\wwwroot\template\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quan.daominh\Documents\HRMv1\ncc-erp-hrm-v2\aspnet-core\src\HRMv2.Web.Host\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C0564F8-9DA4-4B48-9EFB-B99B8C0AFB32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE19D61-DD7A-4130-BB2F-49C1D2DF7CF5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="72">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="77" uniqueCount="75">
   <si>
     <t>Sex</t>
   </si>
@@ -413,6 +413,15 @@
   </si>
   <si>
     <t>Avatar</t>
+  </si>
+  <si>
+    <t>Be Staff From Date</t>
+  </si>
+  <si>
+    <t>Be Tviec From Date</t>
+  </si>
+  <si>
+    <t>MezonUserId</t>
   </si>
 </sst>
 </file>
@@ -526,7 +535,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -566,6 +575,12 @@
     </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -782,7 +797,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AC1"/>
+  <dimension ref="A1:AF1"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="3" width="39.28515625" customWidth="1"/>
@@ -811,9 +826,12 @@
     <col min="27" max="27" width="60.85546875" style="7" customWidth="1"/>
     <col min="28" max="28" width="17.5703125" customWidth="1"/>
     <col min="29" max="29" width="99.5703125" customWidth="1"/>
+    <col min="30" max="30" width="26.42578125" style="8" customWidth="1"/>
+    <col min="31" max="31" width="28.28515625" style="8" customWidth="1"/>
+    <col min="32" max="32" width="22.42578125" style="21" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="14" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:32" s="14" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="10" t="s">
         <v>45</v>
       </c>
@@ -900,6 +918,15 @@
       </c>
       <c r="AC1" s="18" t="s">
         <v>71</v>
+      </c>
+      <c r="AD1" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="AE1" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="AF1" s="10" t="s">
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update : format excel, create User contain mezon user id
</commit_message>
<xml_diff>
--- a/aspnet-core/src/HRMv2.Web.Host/wwwroot/template/Create-Employees.xlsx
+++ b/aspnet-core/src/HRMv2.Web.Host/wwwroot/template/Create-Employees.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\quan.daominh\Documents\HRMv1\ncc-erp-hrm-v2\aspnet-core\src\HRMv2.Web.Host\wwwroot\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EEE19D61-DD7A-4130-BB2F-49C1D2DF7CF5}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75B173FC-D0E6-4402-AD87-7C37C391BF73}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -535,7 +535,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -579,7 +579,10 @@
     <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
   </cellXfs>
@@ -828,7 +831,7 @@
     <col min="29" max="29" width="99.5703125" customWidth="1"/>
     <col min="30" max="30" width="26.42578125" style="8" customWidth="1"/>
     <col min="31" max="31" width="28.28515625" style="8" customWidth="1"/>
-    <col min="32" max="32" width="22.42578125" style="21" customWidth="1"/>
+    <col min="32" max="32" width="22.42578125" style="22" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:32" s="14" customFormat="1" ht="48" customHeight="1" x14ac:dyDescent="0.25">
@@ -925,7 +928,7 @@
       <c r="AE1" s="20" t="s">
         <v>73</v>
       </c>
-      <c r="AF1" s="10" t="s">
+      <c r="AF1" s="21" t="s">
         <v>74</v>
       </c>
     </row>

</xml_diff>